<commit_message>
Updated thresholds for germline risk rate component metric
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/component_level_metrics.xlsx
+++ b/profiles/human-primary-snv/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E84F1C7-829C-4635-8F84-514149D87B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A144F0B9-190A-4AB3-A598-37E0126B9401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -2828,16 +2828,16 @@
         <v>18</v>
       </c>
       <c r="E35">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="F35">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="F35">
-        <v>5.4999999999999997E-3</v>
-      </c>
       <c r="G35">
-        <v>3.5000000000000001E-3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="H35">
-        <v>4.4999999999999997E-3</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="I35" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Moved wet lab component metrics and non-bioinformatically-assessed system metrics to Dropbox
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/component_level_metrics.xlsx
+++ b/profiles/human-primary-snv/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A144F0B9-190A-4AB3-A598-37E0126B9401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4954C7-7A7B-43D7-BDD3-920BDE47AFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$68</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="202">
   <si>
     <t>nn_lower</t>
   </si>
@@ -77,30 +77,9 @@
     <t>Number of soft clipped bases for 90th percentile most softclipped reads</t>
   </si>
   <si>
-    <t>ex_fragmented_DNA_yield</t>
-  </si>
-  <si>
-    <t>ex_tape_station_peak</t>
-  </si>
-  <si>
-    <t>ex_tape_station_area</t>
-  </si>
-  <si>
-    <t>ms_tape_station_peak</t>
-  </si>
-  <si>
-    <t>ms_tape_station_area</t>
-  </si>
-  <si>
     <t>Sample</t>
   </si>
   <si>
-    <t>Batch</t>
-  </si>
-  <si>
-    <t>ex_fragmented_DNA_yield_variability</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -116,48 +95,9 @@
     <t>Name</t>
   </si>
   <si>
-    <t>extracted_DNA_yield</t>
-  </si>
-  <si>
-    <t>extracted_DNA_yield_variability</t>
-  </si>
-  <si>
-    <t>ex_amplified_DNA_yield_variability</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) after enzymatic fragmentation</t>
-  </si>
-  <si>
-    <t>ex_amplified_DNA_conc</t>
-  </si>
-  <si>
-    <t>Concentration (ng/ul) of PCR amplified library. Assumes 20ul elution volume.</t>
-  </si>
-  <si>
-    <t>ms_fragmented_DNA_yield_variability</t>
-  </si>
-  <si>
-    <t>ms_fragmented_DNA_yield</t>
-  </si>
-  <si>
-    <t>ms_ligated_DNA_yield</t>
-  </si>
-  <si>
-    <t>ms_ligated_DNA_yield_variability</t>
-  </si>
-  <si>
     <t>coverage_overlap_ex_ms</t>
   </si>
   <si>
-    <t>DNA extraction</t>
-  </si>
-  <si>
-    <t>EX library preparation</t>
-  </si>
-  <si>
-    <t>MS library preparation</t>
-  </si>
-  <si>
     <t>EX alignment</t>
   </si>
   <si>
@@ -179,9 +119,6 @@
     <t>EX create DSC</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>combined_mask_coverage</t>
   </si>
   <si>
@@ -200,12 +137,6 @@
     <t>ex_insert_size_initial_alignment</t>
   </si>
   <si>
-    <t>Mean length of the largest peak on the tape station report prior to sequencing</t>
-  </si>
-  <si>
-    <t>Integrated area of the largest peak on the tape station report prior to sequencing</t>
-  </si>
-  <si>
     <t>ms_filtered_overrepresented_sequences_r1</t>
   </si>
   <si>
@@ -467,15 +398,6 @@
     <t>ms_coverage_at_depth_threshold</t>
   </si>
   <si>
-    <t>Variability in DNA extraction yield (normalised interquartile range)</t>
-  </si>
-  <si>
-    <t>Variability in DNA quantity post fragmentation (normalised interquartile range)</t>
-  </si>
-  <si>
-    <t>Variability in DNA quantity post adaptor ligation (normalised interquartile range)</t>
-  </si>
-  <si>
     <t>pct_coverage_min_depth</t>
   </si>
   <si>
@@ -536,33 +458,6 @@
     <t>Percentage of reads lost between start and end of EX pipeline</t>
   </si>
   <si>
-    <t>ex_fragmented_DNA_size_pct</t>
-  </si>
-  <si>
-    <t>ex_fragmented_DNA_size_median</t>
-  </si>
-  <si>
-    <t>Percentage of fragments that fall within the expected size range on gel (80-250 bp)</t>
-  </si>
-  <si>
-    <t>ex_amplified_DNA_size_pct</t>
-  </si>
-  <si>
-    <t>ex_amplified_DNA_size_median</t>
-  </si>
-  <si>
-    <t>Percentage of fragments that fall within the expected size range on gel (450-790 bp)</t>
-  </si>
-  <si>
-    <t>Median length of fragments on gel following fragmentation and size selection</t>
-  </si>
-  <si>
-    <t>Median length of fragments on gel following amplification</t>
-  </si>
-  <si>
-    <t>extracted_DNA_size_pct</t>
-  </si>
-  <si>
     <t>EX.MET_SOFTCLIPPING</t>
   </si>
   <si>
@@ -693,18 +588,6 @@
   </si>
   <si>
     <t>germline_risk_rate.value</t>
-  </si>
-  <si>
-    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (&gt;=10,000 bp)</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) required to run assay &amp; QC (ng/uL concentration x uL sample)</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) after enzymatic fragmentation (ng/uL concentration x uL sample)</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) after adaptor ligation (ng/uL concentration x uL sample)</t>
   </si>
   <si>
     <t>Total raw reads obtained from standard Illumina sequencing (6 samples in 3B lane of NovaSeqX)</t>
@@ -1629,7 +1512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -1644,16 +1527,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1668,756 +1551,774 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J1" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="K1" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>220</v>
+        <v>184</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2">
-        <v>2500</v>
+        <v>13</v>
+      </c>
+      <c r="E2" s="1">
+        <v>400000000</v>
       </c>
       <c r="F2" t="s">
         <v>5</v>
       </c>
+      <c r="G2" s="1">
+        <v>500000000</v>
+      </c>
+      <c r="H2" t="s">
+        <v>5</v>
+      </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="K2" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>184</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1">
+        <v>400000000</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="1">
+        <v>500000000</v>
+      </c>
+      <c r="H3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="s">
         <v>143</v>
       </c>
-      <c r="C3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0.52</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0.2</v>
-      </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
-        <v>47</v>
-      </c>
       <c r="K3" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>219</v>
+        <v>116</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E4">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="F4">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G4">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="H4">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="K4" t="s">
-        <v>47</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>221</v>
+        <v>117</v>
       </c>
       <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>35</v>
+      </c>
+      <c r="F5">
+        <v>40</v>
+      </c>
+      <c r="G5">
         <v>39</v>
       </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5">
-        <v>86.2</v>
-      </c>
-      <c r="F5">
-        <v>1000</v>
+      <c r="H5">
+        <v>40</v>
       </c>
       <c r="I5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="K5" t="s">
-        <v>47</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>0.3</v>
+        <v>10</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0.2</v>
+        <v>5</v>
       </c>
       <c r="I6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>222</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E7">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>1000</v>
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="K7" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F8">
-        <v>0.3</v>
+        <v>150</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H8">
-        <v>0.2</v>
+        <v>150</v>
       </c>
       <c r="I8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="K8" t="s">
-        <v>47</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E9">
-        <v>280</v>
+        <v>150</v>
       </c>
       <c r="F9">
-        <v>375.5</v>
+        <v>150</v>
       </c>
       <c r="G9">
-        <v>290</v>
+        <v>150</v>
       </c>
       <c r="H9">
-        <v>310</v>
+        <v>150</v>
       </c>
       <c r="I9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="K9" t="s">
-        <v>47</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>185</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E10">
-        <v>87.9</v>
+        <v>30</v>
       </c>
       <c r="F10">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G10">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="H10">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>47</v>
+        <v>144</v>
       </c>
       <c r="K10" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>223</v>
+        <v>185</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="1">
-        <v>400000000</v>
-      </c>
-      <c r="F11" t="s">
-        <v>5</v>
-      </c>
-      <c r="G11" s="1">
-        <v>500000000</v>
-      </c>
-      <c r="H11" t="s">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="E11">
+        <v>30</v>
+      </c>
+      <c r="F11">
+        <v>40</v>
+      </c>
+      <c r="G11">
+        <v>35</v>
+      </c>
+      <c r="H11">
+        <v>40</v>
       </c>
       <c r="I11" t="b">
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="K11" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>223</v>
+        <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="1">
-        <v>400000000</v>
-      </c>
-      <c r="F12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G12" s="1">
-        <v>500000000</v>
-      </c>
-      <c r="H12" t="s">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0.1</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="K12" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E13">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="I13" t="b">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="K13" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E14">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G14">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I14" t="b">
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="K14" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>138</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
       <c r="F15">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G15">
         <v>0</v>
       </c>
       <c r="H15">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="K15" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E16">
         <v>0</v>
       </c>
       <c r="F16">
+        <v>20</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
         <v>10</v>
       </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>5</v>
-      </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="K16" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
         <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E17">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="G17">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
       <c r="K17" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E18">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G18">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="K18" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>132</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
-        <v>224</v>
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="D19" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G19">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>179</v>
+        <v>145</v>
       </c>
       <c r="K19" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
-        <v>224</v>
+        <v>186</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E20">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="F20">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="G20">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="H20">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="I20" t="b">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>180</v>
+        <v>146</v>
       </c>
       <c r="K20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>187</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H21">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I21" t="b">
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="K21" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>170</v>
       </c>
       <c r="B22" t="s">
-        <v>92</v>
+        <v>188</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D22" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G22">
         <v>0</v>
       </c>
       <c r="H22">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="I22" t="b">
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="K22" t="s">
-        <v>109</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>30</v>
+        <v>0.17</v>
       </c>
       <c r="G23">
         <v>0</v>
       </c>
       <c r="H23">
-        <v>20</v>
+        <v>0.03</v>
       </c>
       <c r="I23" t="b">
         <v>1</v>
@@ -2426,33 +2327,33 @@
         <v>179</v>
       </c>
       <c r="K23" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>189</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D24" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>21.75</v>
       </c>
       <c r="F24">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H24">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="I24" t="b">
         <v>1</v>
@@ -2461,231 +2362,231 @@
         <v>180</v>
       </c>
       <c r="K24" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>190</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D25" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="F25">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="H25">
-        <v>10</v>
+        <v>160</v>
       </c>
       <c r="I25" t="b">
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>179</v>
+        <v>148</v>
       </c>
       <c r="K25" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>181</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>191</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="F26">
-        <v>20</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="H26">
-        <v>10</v>
+        <v>2.0999999999999999E-3</v>
       </c>
       <c r="I26" t="b">
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K26" t="s">
-        <v>111</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>141</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F27">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H27">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="I27" t="b">
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
       <c r="K27" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="D28" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F28">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H28">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I28" t="b">
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="K28" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>150</v>
+        <v>48</v>
       </c>
       <c r="B29" t="s">
-        <v>225</v>
+        <v>117</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="D29" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E29">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="F29">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="G29">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="H29">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="I29" t="b">
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="K29" t="s">
-        <v>128</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="B30" t="s">
-        <v>226</v>
+        <v>115</v>
       </c>
       <c r="C30" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D30" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E30">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F30">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G30">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I30" t="b">
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="K30" t="s">
-        <v>118</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>205</v>
+        <v>50</v>
       </c>
       <c r="B31" t="s">
-        <v>227</v>
+        <v>115</v>
       </c>
       <c r="C31" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D31" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2703,523 +2604,535 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>206</v>
+        <v>166</v>
       </c>
       <c r="K31" t="s">
-        <v>207</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="C32" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D32" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F32">
-        <v>0.17</v>
+        <v>150</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H32">
-        <v>0.03</v>
+        <v>150</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>214</v>
+        <v>165</v>
       </c>
       <c r="K32" t="s">
-        <v>137</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>142</v>
+        <v>55</v>
       </c>
       <c r="B33" t="s">
-        <v>228</v>
+        <v>45</v>
       </c>
       <c r="C33" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D33" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E33">
-        <v>21.75</v>
+        <v>150</v>
       </c>
       <c r="F33">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G33">
-        <v>26.1</v>
+        <v>150</v>
       </c>
       <c r="H33">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I33" t="b">
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>215</v>
+        <v>166</v>
       </c>
       <c r="K33" t="s">
-        <v>146</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="B34" t="s">
-        <v>229</v>
+        <v>192</v>
       </c>
       <c r="C34" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>18</v>
-      </c>
-      <c r="E34">
-        <v>125</v>
-      </c>
-      <c r="F34">
-        <v>175</v>
-      </c>
-      <c r="G34">
-        <v>140</v>
-      </c>
-      <c r="H34">
-        <v>160</v>
+        <v>29</v>
+      </c>
+      <c r="E34" s="1">
+        <v>2850000000</v>
+      </c>
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G34" s="1">
+        <v>3000000000</v>
+      </c>
+      <c r="H34" t="s">
+        <v>5</v>
       </c>
       <c r="I34" t="b">
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="K34" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>216</v>
+        <v>57</v>
       </c>
       <c r="B35" t="s">
-        <v>230</v>
+        <v>192</v>
       </c>
       <c r="C35" t="s">
-        <v>147</v>
+        <v>21</v>
       </c>
       <c r="D35" t="s">
-        <v>18</v>
-      </c>
-      <c r="E35">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="F35">
-        <v>2.5000000000000001E-3</v>
-      </c>
-      <c r="G35">
-        <v>1.6999999999999999E-3</v>
-      </c>
-      <c r="H35">
-        <v>2.0999999999999999E-3</v>
+        <v>29</v>
+      </c>
+      <c r="E35" s="1">
+        <v>2850000000</v>
+      </c>
+      <c r="F35" t="s">
+        <v>5</v>
+      </c>
+      <c r="G35" s="1">
+        <v>3000000000</v>
+      </c>
+      <c r="H35" t="s">
+        <v>5</v>
       </c>
       <c r="I35" t="b">
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>217</v>
+        <v>166</v>
       </c>
       <c r="K35" t="s">
-        <v>218</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>107</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>185</v>
       </c>
       <c r="C36" t="s">
-        <v>147</v>
+        <v>21</v>
       </c>
       <c r="D36" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E36">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F36">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="G36">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="H36">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="I36" t="b">
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>184</v>
+        <v>150</v>
       </c>
       <c r="K36" t="s">
-        <v>122</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>13</v>
+        <v>108</v>
       </c>
       <c r="B37" t="s">
-        <v>29</v>
+        <v>185</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D37" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E37">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="F37">
-        <v>1000</v>
+        <v>40</v>
+      </c>
+      <c r="G37">
+        <v>35</v>
+      </c>
+      <c r="H37">
+        <v>40</v>
       </c>
       <c r="I37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="K37" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D38" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E38">
         <v>0</v>
       </c>
       <c r="F38">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="K38" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>166</v>
+        <v>59</v>
       </c>
       <c r="B39" t="s">
-        <v>168</v>
+        <v>66</v>
       </c>
       <c r="C39" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D39" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E39">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="F39">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="I39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="K39" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>167</v>
+        <v>60</v>
       </c>
       <c r="B40" t="s">
-        <v>172</v>
+        <v>67</v>
       </c>
       <c r="C40" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D40" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E40">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="F40">
+        <v>30</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>20</v>
+      </c>
+      <c r="I40" t="b">
+        <v>1</v>
+      </c>
+      <c r="J40" t="s">
         <v>150</v>
       </c>
-      <c r="G40">
-        <v>120</v>
-      </c>
-      <c r="H40">
-        <v>140</v>
-      </c>
-      <c r="I40" t="b">
-        <v>0</v>
-      </c>
-      <c r="J40" t="s">
-        <v>47</v>
-      </c>
       <c r="K40" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
         <v>30</v>
       </c>
-      <c r="B41" t="s">
-        <v>31</v>
-      </c>
-      <c r="C41" t="s">
-        <v>38</v>
-      </c>
-      <c r="D41" t="s">
-        <v>18</v>
-      </c>
-      <c r="E41">
-        <v>4.3</v>
-      </c>
-      <c r="F41" t="s">
-        <v>5</v>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>20</v>
       </c>
       <c r="I41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="K41" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="B42" t="s">
-        <v>144</v>
+        <v>68</v>
       </c>
       <c r="C42" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D42" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E42">
         <v>0</v>
       </c>
       <c r="F42">
-        <v>0.4</v>
+        <v>20</v>
       </c>
       <c r="G42">
         <v>0</v>
       </c>
       <c r="H42">
-        <v>0.3</v>
+        <v>10</v>
       </c>
       <c r="I42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="K42" t="s">
-        <v>47</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>169</v>
+        <v>63</v>
       </c>
       <c r="B43" t="s">
-        <v>171</v>
+        <v>68</v>
       </c>
       <c r="C43" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D43" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E43">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F43">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="G43">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H43">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="K43" t="s">
-        <v>47</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>170</v>
+        <v>64</v>
       </c>
       <c r="B44" t="s">
-        <v>173</v>
+        <v>118</v>
       </c>
       <c r="C44" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D44" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E44">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="F44">
-        <v>740</v>
+        <v>10</v>
       </c>
       <c r="G44">
-        <v>530</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>650</v>
+        <v>5</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="K44" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>118</v>
       </c>
       <c r="C45" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D45" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E45">
-        <v>544</v>
+        <v>0</v>
       </c>
       <c r="F45">
-        <v>624</v>
+        <v>10</v>
       </c>
       <c r="G45">
-        <v>564</v>
+        <v>0</v>
       </c>
       <c r="H45">
-        <v>604</v>
+        <v>5</v>
       </c>
       <c r="I45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="K45" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B46" t="s">
-        <v>55</v>
+        <v>112</v>
       </c>
       <c r="C46" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="D46" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E46">
-        <v>94.9</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G46">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>47</v>
+        <v>152</v>
       </c>
       <c r="K46" t="s">
-        <v>47</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -3227,1432 +3140,767 @@
         <v>70</v>
       </c>
       <c r="B47" t="s">
-        <v>139</v>
+        <v>193</v>
       </c>
       <c r="C47" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="D47" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E47">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="G47">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>40</v>
+        <v>0.05</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>200</v>
+        <v>152</v>
       </c>
       <c r="K47" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="D48" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E48">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="F48">
         <v>40</v>
       </c>
       <c r="G48">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="H48">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="K48" t="s">
-        <v>105</v>
+        <v>168</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="B49" t="s">
-        <v>138</v>
+        <v>194</v>
       </c>
       <c r="C49" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="D49" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E49">
         <v>0</v>
       </c>
       <c r="F49">
+        <v>20</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
         <v>10</v>
       </c>
-      <c r="G49">
-        <v>0</v>
-      </c>
-      <c r="H49">
-        <v>5</v>
-      </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>200</v>
+        <v>167</v>
       </c>
       <c r="K49" t="s">
-        <v>107</v>
+        <v>169</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="B50" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="C50" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F50">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="G50">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H50">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>201</v>
+        <v>153</v>
       </c>
       <c r="K50" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="C51" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="D51" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E51">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="F51">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G51">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="H51">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>200</v>
+        <v>154</v>
       </c>
       <c r="K51" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>78</v>
+        <v>173</v>
       </c>
       <c r="B52" t="s">
-        <v>68</v>
+        <v>176</v>
       </c>
       <c r="C52" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="D52" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E52">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F52">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G52">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H52">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>201</v>
+        <v>174</v>
       </c>
       <c r="K52" t="s">
-        <v>108</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="B53" t="s">
-        <v>231</v>
+        <v>42</v>
       </c>
       <c r="C53" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="D53" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53">
         <v>50</v>
       </c>
-      <c r="E53" s="1">
-        <v>2850000000</v>
-      </c>
-      <c r="F53" t="s">
-        <v>5</v>
-      </c>
-      <c r="G53" s="1">
-        <v>3000000000</v>
-      </c>
-      <c r="H53" t="s">
-        <v>5</v>
+      <c r="F53">
+        <v>100</v>
+      </c>
+      <c r="G53">
+        <v>75</v>
+      </c>
+      <c r="H53">
+        <v>100</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>200</v>
+        <v>154</v>
       </c>
       <c r="K53" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="B54" t="s">
-        <v>231</v>
+        <v>71</v>
       </c>
       <c r="C54" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="D54" t="s">
-        <v>50</v>
-      </c>
-      <c r="E54" s="1">
-        <v>2850000000</v>
-      </c>
-      <c r="F54" t="s">
-        <v>5</v>
-      </c>
-      <c r="G54" s="1">
-        <v>3000000000</v>
-      </c>
-      <c r="H54" t="s">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="E54">
+        <v>120</v>
+      </c>
+      <c r="F54">
+        <v>180</v>
+      </c>
+      <c r="G54">
+        <v>140</v>
+      </c>
+      <c r="H54">
+        <v>160</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>201</v>
+        <v>155</v>
       </c>
       <c r="K54" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>130</v>
+        <v>78</v>
       </c>
       <c r="B55" t="s">
-        <v>224</v>
+        <v>195</v>
       </c>
       <c r="C55" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D55" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E55">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F55">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="G55">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H55">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="K55" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B56" t="s">
-        <v>224</v>
+        <v>101</v>
       </c>
       <c r="C56" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D56" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E56">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F56">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G56">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="H56">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>186</v>
+        <v>157</v>
       </c>
       <c r="K56" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B57" t="s">
-        <v>89</v>
+        <v>196</v>
       </c>
       <c r="C57" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D57" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H57">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>185</v>
+        <v>158</v>
       </c>
       <c r="K57" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>82</v>
+        <v>175</v>
       </c>
       <c r="B58" t="s">
-        <v>89</v>
+        <v>177</v>
       </c>
       <c r="C58" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D58" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E58">
         <v>0</v>
       </c>
       <c r="F58">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G58">
         <v>0</v>
       </c>
       <c r="H58">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="K58" t="s">
-        <v>109</v>
+        <v>172</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>197</v>
       </c>
       <c r="C59" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D59" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E59">
         <v>0</v>
       </c>
       <c r="F59">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G59">
         <v>0</v>
       </c>
       <c r="H59">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>185</v>
+        <v>158</v>
       </c>
       <c r="K59" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>84</v>
+        <v>136</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>198</v>
       </c>
       <c r="C60" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D60" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E60">
-        <v>0</v>
-      </c>
-      <c r="F60">
-        <v>30</v>
-      </c>
-      <c r="G60">
-        <v>0</v>
-      </c>
-      <c r="H60">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="F60" t="s">
+        <v>5</v>
       </c>
       <c r="I60" t="b">
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>186</v>
+        <v>164</v>
       </c>
       <c r="K60" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="C61" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D61" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E61">
         <v>0</v>
       </c>
       <c r="F61">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="K61" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>86</v>
+        <v>138</v>
       </c>
       <c r="B62" t="s">
-        <v>91</v>
+        <v>199</v>
       </c>
       <c r="C62" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D62" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="F62">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="G62">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H62">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>186</v>
+        <v>141</v>
       </c>
       <c r="K62" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="B63" t="s">
-        <v>141</v>
+        <v>9</v>
       </c>
       <c r="C63" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D63" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
-        <v>10</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G63">
-        <v>0</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H63">
-        <v>5</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="K63" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>88</v>
+        <v>130</v>
       </c>
       <c r="B64" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C64" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D64" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F64">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="G64">
-        <v>0</v>
+        <v>82.8</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="K64" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="B65" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="C65" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="D65" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E65">
         <v>0</v>
       </c>
       <c r="F65">
-        <v>25</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H65">
-        <v>10</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>187</v>
+        <v>161</v>
       </c>
       <c r="K65" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="B66" t="s">
-        <v>232</v>
+        <v>200</v>
       </c>
       <c r="C66" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="D66" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F66">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H66">
-        <v>0.05</v>
+        <v>100</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
       <c r="K66" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B67" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="C67" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="D67" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F67">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H67">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="K67" t="s">
-        <v>203</v>
+        <v>98</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>19</v>
       </c>
       <c r="B68" t="s">
-        <v>233</v>
+        <v>201</v>
       </c>
       <c r="C68" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="D68" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F68">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="G68">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H68">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>202</v>
+        <v>163</v>
       </c>
       <c r="K68" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>148</v>
-      </c>
-      <c r="B69" t="s">
-        <v>149</v>
-      </c>
-      <c r="C69" t="s">
-        <v>43</v>
-      </c>
-      <c r="D69" t="s">
-        <v>18</v>
-      </c>
-      <c r="E69">
-        <v>70</v>
-      </c>
-      <c r="F69">
-        <v>99</v>
-      </c>
-      <c r="G69">
-        <v>85</v>
-      </c>
-      <c r="H69">
-        <v>99</v>
-      </c>
-      <c r="I69" t="b">
-        <v>1</v>
-      </c>
-      <c r="J69" t="s">
-        <v>188</v>
-      </c>
-      <c r="K69" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>52</v>
-      </c>
-      <c r="B70" t="s">
-        <v>64</v>
-      </c>
-      <c r="C70" t="s">
-        <v>40</v>
-      </c>
-      <c r="D70" t="s">
-        <v>18</v>
-      </c>
-      <c r="E70">
-        <v>90</v>
-      </c>
-      <c r="F70">
-        <v>100</v>
-      </c>
-      <c r="G70">
-        <v>95</v>
-      </c>
-      <c r="H70">
-        <v>100</v>
-      </c>
-      <c r="I70" t="b">
-        <v>1</v>
-      </c>
-      <c r="J70" t="s">
-        <v>189</v>
-      </c>
-      <c r="K70" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>208</v>
-      </c>
-      <c r="B71" t="s">
-        <v>211</v>
-      </c>
-      <c r="C71" t="s">
-        <v>40</v>
-      </c>
-      <c r="D71" t="s">
-        <v>18</v>
-      </c>
-      <c r="E71">
-        <v>0</v>
-      </c>
-      <c r="F71">
-        <v>10</v>
-      </c>
-      <c r="G71">
-        <v>0</v>
-      </c>
-      <c r="H71">
-        <v>5</v>
-      </c>
-      <c r="I71" t="b">
-        <v>1</v>
-      </c>
-      <c r="J71" t="s">
-        <v>209</v>
-      </c>
-      <c r="K71" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>51</v>
-      </c>
-      <c r="B72" t="s">
-        <v>65</v>
-      </c>
-      <c r="C72" t="s">
-        <v>40</v>
-      </c>
-      <c r="D72" t="s">
-        <v>18</v>
-      </c>
-      <c r="E72">
-        <v>50</v>
-      </c>
-      <c r="F72">
-        <v>100</v>
-      </c>
-      <c r="G72">
-        <v>75</v>
-      </c>
-      <c r="H72">
-        <v>100</v>
-      </c>
-      <c r="I72" t="b">
-        <v>1</v>
-      </c>
-      <c r="J72" t="s">
-        <v>189</v>
-      </c>
-      <c r="K72" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>53</v>
-      </c>
-      <c r="B73" t="s">
-        <v>94</v>
-      </c>
-      <c r="C73" t="s">
-        <v>40</v>
-      </c>
-      <c r="D73" t="s">
-        <v>18</v>
-      </c>
-      <c r="E73">
-        <v>120</v>
-      </c>
-      <c r="F73">
-        <v>180</v>
-      </c>
-      <c r="G73">
-        <v>140</v>
-      </c>
-      <c r="H73">
-        <v>160</v>
-      </c>
-      <c r="I73" t="b">
-        <v>1</v>
-      </c>
-      <c r="J73" t="s">
-        <v>190</v>
-      </c>
-      <c r="K73" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>101</v>
-      </c>
-      <c r="B74" t="s">
-        <v>234</v>
-      </c>
-      <c r="C74" t="s">
-        <v>46</v>
-      </c>
-      <c r="D74" t="s">
-        <v>18</v>
-      </c>
-      <c r="E74">
-        <v>50</v>
-      </c>
-      <c r="F74">
-        <v>70</v>
-      </c>
-      <c r="G74">
-        <v>50</v>
-      </c>
-      <c r="H74">
-        <v>60</v>
-      </c>
-      <c r="I74" t="b">
-        <v>1</v>
-      </c>
-      <c r="J74" t="s">
-        <v>191</v>
-      </c>
-      <c r="K74" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>154</v>
-      </c>
-      <c r="B75" t="s">
-        <v>124</v>
-      </c>
-      <c r="C75" t="s">
-        <v>46</v>
-      </c>
-      <c r="D75" t="s">
-        <v>18</v>
-      </c>
-      <c r="E75">
-        <v>50</v>
-      </c>
-      <c r="F75">
-        <v>100</v>
-      </c>
-      <c r="G75">
-        <v>90</v>
-      </c>
-      <c r="H75">
-        <v>100</v>
-      </c>
-      <c r="I75" t="b">
-        <v>1</v>
-      </c>
-      <c r="J75" t="s">
-        <v>192</v>
-      </c>
-      <c r="K75" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>99</v>
-      </c>
-      <c r="B76" t="s">
-        <v>235</v>
-      </c>
-      <c r="C76" t="s">
-        <v>46</v>
-      </c>
-      <c r="D76" t="s">
-        <v>18</v>
-      </c>
-      <c r="E76">
-        <v>99</v>
-      </c>
-      <c r="F76">
-        <v>100</v>
-      </c>
-      <c r="G76">
-        <v>99.5</v>
-      </c>
-      <c r="H76">
-        <v>100</v>
-      </c>
-      <c r="I76" t="b">
-        <v>1</v>
-      </c>
-      <c r="J76" t="s">
-        <v>193</v>
-      </c>
-      <c r="K76" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>210</v>
-      </c>
-      <c r="B77" t="s">
-        <v>212</v>
-      </c>
-      <c r="C77" t="s">
-        <v>46</v>
-      </c>
-      <c r="D77" t="s">
-        <v>18</v>
-      </c>
-      <c r="E77">
-        <v>0</v>
-      </c>
-      <c r="F77">
-        <v>10</v>
-      </c>
-      <c r="G77">
-        <v>0</v>
-      </c>
-      <c r="H77">
-        <v>5</v>
-      </c>
-      <c r="I77" t="b">
-        <v>1</v>
-      </c>
-      <c r="J77" t="s">
-        <v>213</v>
-      </c>
-      <c r="K77" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>98</v>
-      </c>
-      <c r="B78" t="s">
-        <v>236</v>
-      </c>
-      <c r="C78" t="s">
-        <v>46</v>
-      </c>
-      <c r="D78" t="s">
-        <v>18</v>
-      </c>
-      <c r="E78">
-        <v>0</v>
-      </c>
-      <c r="F78">
-        <v>15</v>
-      </c>
-      <c r="G78">
-        <v>0</v>
-      </c>
-      <c r="H78">
-        <v>5</v>
-      </c>
-      <c r="I78" t="b">
-        <v>1</v>
-      </c>
-      <c r="J78" t="s">
-        <v>193</v>
-      </c>
-      <c r="K78" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>162</v>
-      </c>
-      <c r="B79" t="s">
-        <v>237</v>
-      </c>
-      <c r="C79" t="s">
-        <v>46</v>
-      </c>
-      <c r="D79" t="s">
-        <v>18</v>
-      </c>
-      <c r="E79">
-        <v>1</v>
-      </c>
-      <c r="F79" t="s">
-        <v>5</v>
-      </c>
-      <c r="I79" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" t="s">
-        <v>199</v>
-      </c>
-      <c r="K79" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>11</v>
-      </c>
-      <c r="B80" t="s">
-        <v>12</v>
-      </c>
-      <c r="C80" t="s">
-        <v>46</v>
-      </c>
-      <c r="D80" t="s">
-        <v>18</v>
-      </c>
-      <c r="E80">
-        <v>0</v>
-      </c>
-      <c r="F80">
-        <v>0</v>
-      </c>
-      <c r="G80">
-        <v>0</v>
-      </c>
-      <c r="H80">
-        <v>0</v>
-      </c>
-      <c r="I80" t="b">
-        <v>1</v>
-      </c>
-      <c r="J80" t="s">
-        <v>175</v>
-      </c>
-      <c r="K80" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>164</v>
-      </c>
-      <c r="B81" t="s">
-        <v>238</v>
-      </c>
-      <c r="C81" t="s">
-        <v>46</v>
-      </c>
-      <c r="D81" t="s">
-        <v>18</v>
-      </c>
-      <c r="E81">
-        <v>14.5</v>
-      </c>
-      <c r="F81">
-        <v>100</v>
-      </c>
-      <c r="G81">
-        <v>26.1</v>
-      </c>
-      <c r="H81">
-        <v>100</v>
-      </c>
-      <c r="I81" t="b">
-        <v>1</v>
-      </c>
-      <c r="J81" t="s">
-        <v>176</v>
-      </c>
-      <c r="K81" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>8</v>
-      </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
-      <c r="C82" t="s">
-        <v>46</v>
-      </c>
-      <c r="D82" t="s">
-        <v>18</v>
-      </c>
-      <c r="E82">
-        <v>0</v>
-      </c>
-      <c r="F82">
-        <v>1.2E-2</v>
-      </c>
-      <c r="G82">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H82">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>194</v>
-      </c>
-      <c r="K82" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>156</v>
-      </c>
-      <c r="B83" t="s">
-        <v>157</v>
-      </c>
-      <c r="C83" t="s">
-        <v>46</v>
-      </c>
-      <c r="D83" t="s">
-        <v>18</v>
-      </c>
-      <c r="E83">
-        <v>69</v>
-      </c>
-      <c r="F83">
-        <v>120</v>
-      </c>
-      <c r="G83">
-        <v>82.8</v>
-      </c>
-      <c r="H83">
-        <v>120</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>195</v>
-      </c>
-      <c r="K83" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>151</v>
-      </c>
-      <c r="B84" t="s">
-        <v>152</v>
-      </c>
-      <c r="C84" t="s">
-        <v>125</v>
-      </c>
-      <c r="D84" t="s">
-        <v>18</v>
-      </c>
-      <c r="E84">
-        <v>0</v>
-      </c>
-      <c r="F84">
-        <v>5.6599999999999999E-4</v>
-      </c>
-      <c r="G84">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H84">
-        <v>3.2679999999999997E-4</v>
-      </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
-        <v>196</v>
-      </c>
-      <c r="K84" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>10</v>
-      </c>
-      <c r="B85" t="s">
-        <v>239</v>
-      </c>
-      <c r="C85" t="s">
-        <v>125</v>
-      </c>
-      <c r="D85" t="s">
-        <v>18</v>
-      </c>
-      <c r="E85">
-        <v>4</v>
-      </c>
-      <c r="F85">
-        <v>100</v>
-      </c>
-      <c r="G85">
-        <v>20</v>
-      </c>
-      <c r="H85">
-        <v>100</v>
-      </c>
-      <c r="I85" t="b">
-        <v>1</v>
-      </c>
-      <c r="J85" t="s">
-        <v>176</v>
-      </c>
-      <c r="K85" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>155</v>
-      </c>
-      <c r="B86" t="s">
-        <v>165</v>
-      </c>
-      <c r="C86" t="s">
-        <v>125</v>
-      </c>
-      <c r="D86" t="s">
-        <v>18</v>
-      </c>
-      <c r="E86">
-        <v>0</v>
-      </c>
-      <c r="F86">
-        <v>95</v>
-      </c>
-      <c r="G86">
-        <v>0</v>
-      </c>
-      <c r="H86">
-        <v>80</v>
-      </c>
-      <c r="I86" t="b">
-        <v>1</v>
-      </c>
-      <c r="J86" t="s">
-        <v>197</v>
-      </c>
-      <c r="K86" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>36</v>
-      </c>
-      <c r="B87" t="s">
-        <v>240</v>
-      </c>
-      <c r="C87" t="s">
-        <v>125</v>
-      </c>
-      <c r="D87" t="s">
-        <v>18</v>
-      </c>
-      <c r="E87">
-        <v>33</v>
-      </c>
-      <c r="F87">
-        <v>100</v>
-      </c>
-      <c r="G87">
-        <v>67</v>
-      </c>
-      <c r="H87">
-        <v>100</v>
-      </c>
-      <c r="I87" t="b">
-        <v>1</v>
-      </c>
-      <c r="J87" t="s">
-        <v>198</v>
-      </c>
-      <c r="K87" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K87" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K68" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Renamed ex_variant_call eligible component metric to ex_genome_call eligible
</commit_message>
<xml_diff>
--- a/profiles/human-primary-snv/component_level_metrics.xlsx
+++ b/profiles/human-primary-snv/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\profiles\human-primary-snv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4954C7-7A7B-43D7-BDD3-920BDE47AFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ABB0315-3C1E-4AC2-B0BD-CCE68DB0F7A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>Rate at which Watson and Crick complementary bases disagree (total R1R2 disagreements divided by total duplex bases for each sample)</t>
   </si>
   <si>
-    <t>ex_variant_call_eligible</t>
-  </si>
-  <si>
     <t>ex_dsc_softclipping</t>
   </si>
   <si>
@@ -642,6 +639,9 @@
   </si>
   <si>
     <t>Percentage of all sequenced bases with MS depth &gt;= min_depth threshold AND EX duplex depth &gt; 0</t>
+  </si>
+  <si>
+    <t>ex_genome_call_eligible</t>
   </si>
 </sst>
 </file>
@@ -1527,16 +1527,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1551,13 +1551,13 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K1" t="s">
         <v>79</v>
-      </c>
-      <c r="K1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1565,13 +1565,13 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1">
         <v>400000000</v>
@@ -1589,10 +1589,10 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1600,13 +1600,13 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1">
         <v>400000000</v>
@@ -1624,24 +1624,24 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4">
         <v>35</v>
@@ -1659,24 +1659,24 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5">
         <v>35</v>
@@ -1694,24 +1694,24 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1729,24 +1729,24 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1764,24 +1764,24 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8">
         <v>150</v>
@@ -1799,24 +1799,24 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
         <v>44</v>
       </c>
-      <c r="B9" t="s">
-        <v>45</v>
-      </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9">
         <v>150</v>
@@ -1834,24 +1834,24 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10">
         <v>30</v>
@@ -1869,24 +1869,24 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11">
         <v>30</v>
@@ -1904,24 +1904,24 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -1939,24 +1939,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1974,24 +1974,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -2009,24 +2009,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2044,24 +2044,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2079,24 +2079,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -2114,24 +2114,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -2149,24 +2149,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -2184,24 +2184,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20">
         <v>70</v>
@@ -2219,24 +2219,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21">
         <v>90</v>
@@ -2254,24 +2254,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B22" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2289,24 +2289,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
+        <v>170</v>
+      </c>
+      <c r="K22" t="s">
         <v>171</v>
-      </c>
-      <c r="K22" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2324,24 +2324,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E24">
         <v>21.75</v>
@@ -2359,24 +2359,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <v>125</v>
@@ -2394,24 +2394,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B26" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E26">
         <v>1.2999999999999999E-3</v>
@@ -2429,24 +2429,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
+        <v>181</v>
+      </c>
+      <c r="K26" t="s">
         <v>182</v>
-      </c>
-      <c r="K26" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E27">
         <v>70</v>
@@ -2464,24 +2464,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28">
         <v>35</v>
@@ -2499,24 +2499,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E29">
         <v>35</v>
@@ -2534,24 +2534,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -2569,24 +2569,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2604,24 +2604,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E32">
         <v>150</v>
@@ -2639,24 +2639,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E33">
         <v>150</v>
@@ -2674,24 +2674,24 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E34" s="1">
         <v>2850000000</v>
@@ -2709,24 +2709,24 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E35" s="1">
         <v>2850000000</v>
@@ -2744,24 +2744,24 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36">
         <v>30</v>
@@ -2779,24 +2779,24 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E37">
         <v>30</v>
@@ -2814,24 +2814,24 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -2849,24 +2849,24 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E39">
         <v>0</v>
@@ -2884,24 +2884,24 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2919,24 +2919,24 @@
         <v>1</v>
       </c>
       <c r="J40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C41" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -2954,24 +2954,24 @@
         <v>1</v>
       </c>
       <c r="J41" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C42" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D42" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -2989,24 +2989,24 @@
         <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C43" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E43">
         <v>0</v>
@@ -3024,24 +3024,24 @@
         <v>1</v>
       </c>
       <c r="J43" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B44" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C44" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -3059,24 +3059,24 @@
         <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E45">
         <v>0</v>
@@ -3094,24 +3094,24 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K45" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>27</v>
+      </c>
+      <c r="B46" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" t="s">
         <v>28</v>
-      </c>
-      <c r="B46" t="s">
-        <v>112</v>
-      </c>
-      <c r="C46" t="s">
-        <v>23</v>
-      </c>
-      <c r="D46" t="s">
-        <v>29</v>
       </c>
       <c r="E46">
         <v>0</v>
@@ -3129,24 +3129,24 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -3164,24 +3164,24 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>102</v>
+      </c>
+      <c r="B48" t="s">
         <v>103</v>
       </c>
-      <c r="B48" t="s">
-        <v>104</v>
-      </c>
       <c r="C48" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E48">
         <v>1</v>
@@ -3199,24 +3199,24 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
+        <v>166</v>
+      </c>
+      <c r="K48" t="s">
         <v>167</v>
-      </c>
-      <c r="K48" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B49" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C49" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -3234,24 +3234,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K49" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" t="s">
         <v>122</v>
       </c>
-      <c r="B50" t="s">
-        <v>123</v>
-      </c>
       <c r="C50" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E50">
         <v>70</v>
@@ -3269,24 +3269,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K50" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51">
         <v>90</v>
@@ -3304,24 +3304,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K51" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B52" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C52" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -3339,24 +3339,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K52" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B53" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E53">
         <v>50</v>
@@ -3374,24 +3374,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K53" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C54" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E54">
         <v>120</v>
@@ -3409,24 +3409,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K54" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B55" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C55" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E55">
         <v>50</v>
@@ -3444,24 +3444,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K55" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C56" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E56">
         <v>50</v>
@@ -3479,24 +3479,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B57" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C57" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E57">
         <v>99</v>
@@ -3514,24 +3514,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K57" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B58" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C58" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -3549,24 +3549,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K58" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B59" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C59" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3584,24 +3584,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C60" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E60">
         <v>1</v>
@@ -3613,24 +3613,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
         <v>11</v>
       </c>
-      <c r="B61" t="s">
-        <v>12</v>
-      </c>
       <c r="C61" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3648,24 +3648,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B62" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C62" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D62" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E62">
         <v>14.5</v>
@@ -3683,10 +3683,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K62" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3697,10 +3697,10 @@
         <v>9</v>
       </c>
       <c r="C63" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D63" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3718,24 +3718,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K63" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>129</v>
+      </c>
+      <c r="B64" t="s">
         <v>130</v>
       </c>
-      <c r="B64" t="s">
-        <v>131</v>
-      </c>
       <c r="C64" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D64" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E64">
         <v>69</v>
@@ -3753,24 +3753,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K64" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>124</v>
+      </c>
+      <c r="B65" t="s">
         <v>125</v>
       </c>
-      <c r="B65" t="s">
-        <v>126</v>
-      </c>
       <c r="C65" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -3788,24 +3788,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K65" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>10</v>
+        <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C66" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D66" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E66">
         <v>4</v>
@@ -3823,24 +3823,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K66" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C67" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D67" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3858,24 +3858,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K67" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B68" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C68" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D68" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E68">
         <v>33</v>
@@ -3893,10 +3893,10 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K68" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>